<commit_message>
Fix SUI trade #74: Signal=Viona, Account=Bitget
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TOCH_Trading_2026_v2.1.xlsx
+++ b/TOCH_Trading_2026_v2.1.xlsx
@@ -7104,7 +7104,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>HEMI V8_1</t>
+          <t>Viona</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -7119,7 +7119,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>CK_one</t>
+          <t>Bitget</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -7180,8 +7180,6 @@
         </is>
       </c>
     </row>
-    <row r="72"/>
-    <row r="73"/>
     <row r="74">
       <c r="Y74" s="44" t="n"/>
       <c r="Z74" s="44" t="n"/>

</xml_diff>

<commit_message>
Fix trades: add #74 CFX, remove DOGE duplicate, renumber, no gaps
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TOCH_Trading_2026_v2.1.xlsx
+++ b/TOCH_Trading_2026_v2.1.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trades" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistik" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KODA-Bot" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Trades'!$A$1:$AA$61</definedName>
@@ -30,7 +31,7 @@
     <numFmt numFmtId="172" formatCode="#,#00.0%;[Red]\-#,#00.0%"/>
     <numFmt numFmtId="173" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -119,8 +120,14 @@
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0000C8FF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="22">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -227,8 +234,14 @@
         <fgColor rgb="FFC8E6C9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000D1B2E"/>
+        <bgColor rgb="000D1B2E"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -310,11 +323,16 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="001E3A5F"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -497,6 +515,9 @@
     <xf numFmtId="171" fontId="0" fillId="17" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="22" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -863,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB78"/>
+  <dimension ref="A1:AB85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7100,7 +7121,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -7109,84 +7130,311 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>04.05.26</t>
+          <t>27-4-26</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>04:51:00</t>
+          <t>07:09</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Bitget</t>
+          <t>BitGet</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>SUI</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Short</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>2804.0</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>2804.0</t>
-        </is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>1747.3</v>
       </c>
       <c r="J71" t="n">
-        <v>15</v>
-      </c>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t>0.9383</t>
-        </is>
+        <v>11</v>
+      </c>
+      <c r="L71" t="n">
+        <v>19220.32</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0.06022</v>
       </c>
       <c r="T71" t="inlineStr">
         <is>
-          <t>04.05.26</t>
+          <t>27-4-26</t>
         </is>
       </c>
       <c r="U71" t="inlineStr">
         <is>
-          <t>06:32:00</t>
-        </is>
-      </c>
-      <c r="V71" t="inlineStr">
-        <is>
-          <t>0.9254</t>
-        </is>
+          <t>07:14</t>
+        </is>
+      </c>
+      <c r="V71" t="n">
+        <v>0.06027</v>
       </c>
       <c r="W71" s="31" t="n">
-        <v>0.06966435185185185</v>
+        <v>0.003611111111111111</v>
       </c>
       <c r="X71" t="n">
-        <v>18.96</v>
+        <v>-2.01</v>
       </c>
       <c r="Y71" t="n">
-        <v>531.84</v>
+        <v>-13.96</v>
+      </c>
+      <c r="Z71" t="n">
+        <v>-35.04</v>
       </c>
       <c r="AA71" t="inlineStr">
         <is>
           <t>j</t>
         </is>
       </c>
+      <c r="AB71" t="inlineStr">
+        <is>
+          <t>Falsche Eingabe (Short)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Viona</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>27-4-26</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>07:14</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>BitGet</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>SEI</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>1756.78</v>
+      </c>
+      <c r="J72" t="n">
+        <v>11</v>
+      </c>
+      <c r="L72" t="n">
+        <v>19324.54</v>
+      </c>
+      <c r="M72" t="n">
+        <v>0.06028</v>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>27-4-26</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>08:58</t>
+        </is>
+      </c>
+      <c r="V72" t="n">
+        <v>0.06059</v>
+      </c>
+      <c r="W72" s="31" t="n">
+        <v>0.07225694444444444</v>
+      </c>
+      <c r="X72" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="Y72" t="n">
+        <v>98.81</v>
+      </c>
+      <c r="Z72" t="n">
+        <v>75.68000000000001</v>
+      </c>
+      <c r="AA72" t="inlineStr">
+        <is>
+          <t>j</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>22-4-26</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>07:05</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Phemex</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>LTC</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>988.14</v>
+      </c>
+      <c r="J73" t="n">
+        <v>5</v>
+      </c>
+      <c r="L73" t="n">
+        <v>4940.684</v>
+      </c>
+      <c r="M73" t="n">
+        <v>56.24</v>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>26-4-26</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="V73" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="W73" s="31" t="n">
+        <v>4.579861111111111</v>
+      </c>
+      <c r="X73" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="Y73" t="n">
+        <v>22.7664</v>
+      </c>
+      <c r="Z73" t="n">
+        <v>11.3262</v>
+      </c>
+      <c r="AA73" t="inlineStr">
+        <is>
+          <t>j</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="Y74" s="44" t="n"/>
-      <c r="Z74" s="44" t="n"/>
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>29-4-26</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>BitGet</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>DOGE</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>2090.56</v>
+      </c>
+      <c r="J74" t="n">
+        <v>25</v>
+      </c>
+      <c r="L74" t="n">
+        <v>52264.11</v>
+      </c>
+      <c r="M74" t="n">
+        <v>0.10956</v>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>29-4-26</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>08:29</t>
+        </is>
+      </c>
+      <c r="V74" t="n">
+        <v>0.10722</v>
+      </c>
+      <c r="W74" s="31" t="n">
+        <v>0.01994212962962963</v>
+      </c>
+      <c r="X74" t="n">
+        <v>50.69</v>
+      </c>
+      <c r="Y74" s="44" t="n">
+        <v>1146.42</v>
+      </c>
+      <c r="Z74" s="44" t="n">
+        <v>1083.02</v>
+      </c>
+      <c r="AA74" t="inlineStr">
+        <is>
+          <t>j</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -7195,80 +7443,38 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>27-4-26</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>07:09</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>BitGet</t>
+          <t>28-4-26</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>CFX</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="I75" t="n">
-        <v>1747.3</v>
+          <t>L</t>
+        </is>
       </c>
       <c r="J75" t="n">
-        <v>11</v>
-      </c>
-      <c r="L75" t="n">
-        <v>19220.32</v>
-      </c>
-      <c r="M75" t="n">
-        <v>0.06022</v>
-      </c>
-      <c r="T75" t="inlineStr">
-        <is>
-          <t>27-4-26</t>
-        </is>
-      </c>
-      <c r="U75" t="inlineStr">
-        <is>
-          <t>07:14</t>
-        </is>
-      </c>
-      <c r="V75" t="n">
-        <v>0.06027</v>
-      </c>
-      <c r="W75" s="31" t="n">
-        <v>0.003611111111111111</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="W75" s="31" t="n"/>
       <c r="X75" t="n">
-        <v>-2.01</v>
+        <v>20.87</v>
       </c>
       <c r="Y75" t="n">
-        <v>-13.96</v>
-      </c>
-      <c r="Z75" t="n">
-        <v>-35.04</v>
+        <v>208.77</v>
       </c>
       <c r="AA75" t="inlineStr">
         <is>
           <t>j</t>
-        </is>
-      </c>
-      <c r="AB75" t="inlineStr">
-        <is>
-          <t>Falsche Eingabe (Short)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -7277,65 +7483,70 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>27-4-26</t>
+          <t>04.05.26</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>07:14</t>
+          <t>04:51:00</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>BitGet</t>
+          <t>Bitget</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>SUI</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>l</t>
-        </is>
-      </c>
-      <c r="I76" t="n">
-        <v>1756.78</v>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>2804.0</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>2804.0</t>
+        </is>
       </c>
       <c r="J76" t="n">
-        <v>11</v>
-      </c>
-      <c r="L76" t="n">
-        <v>19324.54</v>
-      </c>
-      <c r="M76" t="n">
-        <v>0.06028</v>
+        <v>15</v>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>0.9383</t>
+        </is>
       </c>
       <c r="T76" t="inlineStr">
         <is>
-          <t>27-4-26</t>
+          <t>04.05.26</t>
         </is>
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>08:58</t>
-        </is>
-      </c>
-      <c r="V76" t="n">
-        <v>0.06059</v>
+          <t>06:32:00</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>0.9254</t>
+        </is>
       </c>
       <c r="W76" s="31" t="n">
-        <v>0.07225694444444444</v>
+        <v>0.06966435185185185</v>
       </c>
       <c r="X76" t="n">
-        <v>4.32</v>
+        <v>18.96</v>
       </c>
       <c r="Y76" t="n">
-        <v>98.81</v>
-      </c>
-      <c r="Z76" t="n">
-        <v>75.68000000000001</v>
+        <v>531.84</v>
       </c>
       <c r="AA76" t="inlineStr">
         <is>
@@ -7344,159 +7555,18 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="n">
-        <v>72</v>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>CK</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>22-4-26</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>07:05</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>Phemex</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>LTC</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>l</t>
-        </is>
-      </c>
-      <c r="I77" t="n">
-        <v>988.14</v>
-      </c>
-      <c r="J77" t="n">
-        <v>5</v>
-      </c>
-      <c r="L77" t="n">
-        <v>4940.684</v>
-      </c>
-      <c r="M77" t="n">
-        <v>56.24</v>
-      </c>
-      <c r="T77" t="inlineStr">
-        <is>
-          <t>26-4-26</t>
-        </is>
-      </c>
-      <c r="U77" t="inlineStr">
-        <is>
-          <t>21:00</t>
-        </is>
-      </c>
-      <c r="V77" t="n">
-        <v>56.5</v>
-      </c>
-      <c r="W77" s="31" t="n">
-        <v>4.579861111111111</v>
-      </c>
-      <c r="X77" t="n">
-        <v>2.27</v>
-      </c>
-      <c r="Y77" t="n">
-        <v>22.7664</v>
-      </c>
-      <c r="Z77" t="n">
-        <v>11.3262</v>
-      </c>
-      <c r="AA77" t="inlineStr">
-        <is>
-          <t>j</t>
-        </is>
-      </c>
+      <c r="W77" s="31" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" t="n">
-        <v>73</v>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>CK</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>29-4-26</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>BitGet</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>DOGE</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="I78" t="n">
-        <v>2090.56</v>
-      </c>
-      <c r="J78" t="n">
-        <v>25</v>
-      </c>
-      <c r="L78" t="n">
-        <v>52264.11</v>
-      </c>
-      <c r="M78" t="n">
-        <v>0.10956</v>
-      </c>
-      <c r="T78" t="inlineStr">
-        <is>
-          <t>29-4-26</t>
-        </is>
-      </c>
-      <c r="U78" t="inlineStr">
-        <is>
-          <t>08:29</t>
-        </is>
-      </c>
-      <c r="V78" t="n">
-        <v>0.10722</v>
-      </c>
-      <c r="W78" s="31" t="n">
-        <v>0.01994212962962963</v>
-      </c>
-      <c r="X78" t="n">
-        <v>50.69</v>
-      </c>
-      <c r="Y78" t="n">
-        <v>1146.42</v>
-      </c>
-      <c r="Z78" t="n">
-        <v>1083.02</v>
-      </c>
-      <c r="AA78" t="inlineStr">
-        <is>
-          <t>j</t>
-        </is>
-      </c>
-    </row>
+      <c r="W78" s="31" t="n"/>
+    </row>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
   </sheetData>
   <autoFilter ref="A1:AA61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8834,4 +8904,255 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="66" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="66" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="C1" s="66" t="inlineStr">
+        <is>
+          <t>Zeit</t>
+        </is>
+      </c>
+      <c r="D1" s="66" t="inlineStr">
+        <is>
+          <t>Coin</t>
+        </is>
+      </c>
+      <c r="E1" s="66" t="inlineStr">
+        <is>
+          <t>Richtung</t>
+        </is>
+      </c>
+      <c r="F1" s="66" t="inlineStr">
+        <is>
+          <t>Strategie</t>
+        </is>
+      </c>
+      <c r="G1" s="66" t="inlineStr">
+        <is>
+          <t>Entry</t>
+        </is>
+      </c>
+      <c r="H1" s="66" t="inlineStr">
+        <is>
+          <t>TP1 (50%)</t>
+        </is>
+      </c>
+      <c r="I1" s="66" t="inlineStr">
+        <is>
+          <t>TP1 Kurs</t>
+        </is>
+      </c>
+      <c r="J1" s="66" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="K1" s="66" t="inlineStr">
+        <is>
+          <t>SL Kurs</t>
+        </is>
+      </c>
+      <c r="L1" s="66" t="inlineStr">
+        <is>
+          <t>Rest Exit</t>
+        </is>
+      </c>
+      <c r="M1" s="66" t="inlineStr">
+        <is>
+          <t>Rest Kurs</t>
+        </is>
+      </c>
+      <c r="N1" s="66" t="inlineStr">
+        <is>
+          <t>ROI %</t>
+        </is>
+      </c>
+      <c r="O1" s="66" t="inlineStr">
+        <is>
+          <t>PNL USDT</t>
+        </is>
+      </c>
+      <c r="P1" s="66" t="inlineStr">
+        <is>
+          <t>Net PNL</t>
+        </is>
+      </c>
+      <c r="Q1" s="66" t="inlineStr">
+        <is>
+          <t>Dauer</t>
+        </is>
+      </c>
+      <c r="R1" s="66" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="S1" s="66" t="inlineStr">
+        <is>
+          <t>EE Main</t>
+        </is>
+      </c>
+      <c r="T1" s="66" t="inlineStr">
+        <is>
+          <t>EE Signal</t>
+        </is>
+      </c>
+      <c r="U1" s="66" t="inlineStr">
+        <is>
+          <t>Steilheit %</t>
+        </is>
+      </c>
+      <c r="V1" s="66" t="inlineStr">
+        <is>
+          <t>Golden Wick</t>
+        </is>
+      </c>
+      <c r="W1" s="66" t="inlineStr">
+        <is>
+          <t>Notiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ER1</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>76500</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>+1.0%</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>77265</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>-1.2%</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>75582</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Trailing</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>77800</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>2.5h</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>TESTNET</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="T2" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="U2" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Erster Testnet-Trade</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Sync all: add #73 MarkTrade BTC, renumber #74 DOGE #75 CFX #76 SUI
Excel + all 3 HTML pages now match: 76 trades, no gaps, no duplicates.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TOCH_Trading_2026_v2.1.xlsx
+++ b/TOCH_Trading_2026_v2.1.xlsx
@@ -7361,70 +7361,74 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>CK</t>
+          <t>MarkTrade</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>29-4-26</t>
+          <t>25-4-26</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>13:22:00</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>BitGet</t>
+          <t>Phemex</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>DOGE</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I74" t="n">
-        <v>2090.56</v>
+        <v>414.57</v>
       </c>
       <c r="J74" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="L74" t="n">
-        <v>52264.11</v>
-      </c>
-      <c r="M74" t="n">
-        <v>0.10956</v>
+        <v>20728.46</v>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>77345.0</t>
+        </is>
       </c>
       <c r="T74" t="inlineStr">
         <is>
-          <t>29-4-26</t>
+          <t>27-4-26</t>
         </is>
       </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>08:29</t>
-        </is>
-      </c>
-      <c r="V74" t="n">
-        <v>0.10722</v>
+          <t>11:10:00</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>77404.9</t>
+        </is>
       </c>
       <c r="W74" s="31" t="n">
-        <v>0.01994212962962963</v>
+        <v>1.907638888888889</v>
       </c>
       <c r="X74" t="n">
-        <v>50.69</v>
+        <v>-3.96</v>
       </c>
       <c r="Y74" s="44" t="n">
-        <v>1146.42</v>
+        <v>-16.05</v>
       </c>
       <c r="Z74" s="44" t="n">
-        <v>1083.02</v>
+        <v>-33.35</v>
       </c>
       <c r="AA74" t="inlineStr">
         <is>
@@ -7438,33 +7442,70 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Viona</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>28-4-26</t>
+          <t>29-4-26</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>BitGet</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>CFX</t>
+          <t>DOGE</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>2090.56</v>
       </c>
       <c r="J75" t="n">
-        <v>10</v>
-      </c>
-      <c r="W75" s="31" t="n"/>
+        <v>25</v>
+      </c>
+      <c r="L75" t="n">
+        <v>52264.11</v>
+      </c>
+      <c r="M75" t="n">
+        <v>0.10956</v>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>29-4-26</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>08:29</t>
+        </is>
+      </c>
+      <c r="V75" t="n">
+        <v>0.10722</v>
+      </c>
+      <c r="W75" s="31" t="n">
+        <v>0.01994212962962963</v>
+      </c>
       <c r="X75" t="n">
-        <v>20.87</v>
+        <v>50.69</v>
       </c>
       <c r="Y75" t="n">
-        <v>208.77</v>
+        <v>1146.42</v>
+      </c>
+      <c r="Z75" t="n">
+        <v>1083.02</v>
       </c>
       <c r="AA75" t="inlineStr">
         <is>
@@ -7483,79 +7524,116 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
+          <t>28-4-26</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>CFX</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
+        <v>10</v>
+      </c>
+      <c r="W76" s="31" t="n"/>
+      <c r="X76" t="n">
+        <v>20.87</v>
+      </c>
+      <c r="Y76" t="n">
+        <v>208.77</v>
+      </c>
+      <c r="AA76" t="inlineStr">
+        <is>
+          <t>j</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Viona</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
           <t>04.05.26</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D77" t="inlineStr">
         <is>
           <t>04:51:00</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>Bitget</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F77" t="inlineStr">
         <is>
           <t>SUI</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
+      <c r="G77" t="inlineStr">
         <is>
           <t>Short</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr">
+      <c r="H77" t="inlineStr">
         <is>
           <t>2804.0</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr">
+      <c r="I77" t="inlineStr">
         <is>
           <t>2804.0</t>
         </is>
       </c>
-      <c r="J76" t="n">
+      <c r="J77" t="n">
         <v>15</v>
       </c>
-      <c r="M76" t="inlineStr">
+      <c r="M77" t="inlineStr">
         <is>
           <t>0.9383</t>
         </is>
       </c>
-      <c r="T76" t="inlineStr">
+      <c r="T77" t="inlineStr">
         <is>
           <t>04.05.26</t>
         </is>
       </c>
-      <c r="U76" t="inlineStr">
+      <c r="U77" t="inlineStr">
         <is>
           <t>06:32:00</t>
         </is>
       </c>
-      <c r="V76" t="inlineStr">
+      <c r="V77" t="inlineStr">
         <is>
           <t>0.9254</t>
         </is>
       </c>
-      <c r="W76" s="31" t="n">
+      <c r="W77" s="31" t="n">
         <v>0.06966435185185185</v>
       </c>
-      <c r="X76" t="n">
+      <c r="X77" t="n">
         <v>18.96</v>
       </c>
-      <c r="Y76" t="n">
+      <c r="Y77" t="n">
         <v>531.84</v>
       </c>
-      <c r="AA76" t="inlineStr">
+      <c r="AA77" t="inlineStr">
         <is>
           <t>j</t>
         </is>
       </c>
-    </row>
-    <row r="77">
-      <c r="W77" s="31" t="n"/>
     </row>
     <row r="78">
       <c r="W78" s="31" t="n"/>

</xml_diff>

<commit_message>
Dashboard Update 16.06.2026 03:03
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TOCH_Trading_2026_v2.1.xlsx
+++ b/TOCH_Trading_2026_v2.1.xlsx
@@ -9,6 +9,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trades" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistik" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KODA-Bot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auszahlungen" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boersenstand" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ausgaben" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistik_Calc" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Trades'!$A$1:$AA$61</definedName>
@@ -31,7 +35,7 @@
     <numFmt numFmtId="172" formatCode="#,#00.0%;[Red]\-#,#00.0%"/>
     <numFmt numFmtId="173" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -126,8 +130,16 @@
       <color rgb="0000C8FF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="23">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -240,8 +252,14 @@
         <bgColor rgb="000D1B2E"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
+        <bgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -328,11 +346,17 @@
         <color rgb="001E3A5F"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -519,6 +543,28 @@
     <xf numFmtId="0" fontId="13" fillId="22" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="15" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -884,7 +930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB85"/>
+  <dimension ref="A1:AB78"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7638,13 +7684,6 @@
     <row r="78">
       <c r="W78" s="31" t="n"/>
     </row>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
   </sheetData>
   <autoFilter ref="A1:AA61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9233,4 +9272,811 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0022C55E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="67" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="67" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="C1" s="67" t="inlineStr">
+        <is>
+          <t>Gewinn_Brutto</t>
+        </is>
+      </c>
+      <c r="D1" s="67" t="inlineStr">
+        <is>
+          <t>Ausgaben</t>
+        </is>
+      </c>
+      <c r="E1" s="67" t="inlineStr">
+        <is>
+          <t>Ausgaben_Detail</t>
+        </is>
+      </c>
+      <c r="F1" s="67" t="inlineStr">
+        <is>
+          <t>Verteilung</t>
+        </is>
+      </c>
+      <c r="G1" s="67" t="inlineStr">
+        <is>
+          <t>TR_25pct</t>
+        </is>
+      </c>
+      <c r="H1" s="67" t="inlineStr">
+        <is>
+          <t>GT_25pct</t>
+        </is>
+      </c>
+      <c r="I1" s="67" t="inlineStr">
+        <is>
+          <t>CK_50pct</t>
+        </is>
+      </c>
+      <c r="J1" s="67" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="68" t="inlineStr">
+        <is>
+          <t>31.03.2026</t>
+        </is>
+      </c>
+      <c r="C2" s="69" t="n">
+        <v>1090</v>
+      </c>
+      <c r="D2" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="68" t="inlineStr"/>
+      <c r="F2" s="69">
+        <f>C2+D2</f>
+        <v/>
+      </c>
+      <c r="G2" s="69">
+        <f>F2*0.5</f>
+        <v/>
+      </c>
+      <c r="H2" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="69">
+        <f>F2*0.5</f>
+        <v/>
+      </c>
+      <c r="J2" s="68" t="inlineStr">
+        <is>
+          <t>Ausbezahlt</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="68" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="68" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C3" s="69" t="n">
+        <v>866</v>
+      </c>
+      <c r="D3" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="68" t="inlineStr"/>
+      <c r="F3" s="69">
+        <f>C3+D3</f>
+        <v/>
+      </c>
+      <c r="G3" s="69">
+        <f>F3*0.5</f>
+        <v/>
+      </c>
+      <c r="H3" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="69">
+        <f>F3*0.5</f>
+        <v/>
+      </c>
+      <c r="J3" s="68" t="inlineStr">
+        <is>
+          <t>Ausbezahlt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="68" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="68" t="inlineStr">
+        <is>
+          <t>09.04.2026</t>
+        </is>
+      </c>
+      <c r="C4" s="69" t="n">
+        <v>426</v>
+      </c>
+      <c r="D4" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="68" t="inlineStr"/>
+      <c r="F4" s="69">
+        <f>C4+D4</f>
+        <v/>
+      </c>
+      <c r="G4" s="69">
+        <f>F4*0.5</f>
+        <v/>
+      </c>
+      <c r="H4" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="69">
+        <f>F4*0.5</f>
+        <v/>
+      </c>
+      <c r="J4" s="68" t="inlineStr">
+        <is>
+          <t>Ausbezahlt</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="68" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="68" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="C5" s="69" t="n">
+        <v>2350</v>
+      </c>
+      <c r="D5" s="69" t="n">
+        <v>-100</v>
+      </c>
+      <c r="E5" s="68" t="inlineStr">
+        <is>
+          <t>Claude Code Abo</t>
+        </is>
+      </c>
+      <c r="F5" s="69">
+        <f>C5+D5</f>
+        <v/>
+      </c>
+      <c r="G5" s="69">
+        <f>F5*0.25</f>
+        <v/>
+      </c>
+      <c r="H5" s="69">
+        <f>F5*0.25</f>
+        <v/>
+      </c>
+      <c r="I5" s="69">
+        <f>F5*0.50</f>
+        <v/>
+      </c>
+      <c r="J5" s="68" t="inlineStr">
+        <is>
+          <t>Ausbezahlt</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="68" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="68" t="inlineStr">
+        <is>
+          <t>12.05.2026</t>
+        </is>
+      </c>
+      <c r="C6" s="69" t="n">
+        <v>2983</v>
+      </c>
+      <c r="D6" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="68" t="inlineStr"/>
+      <c r="F6" s="69">
+        <f>C6+D6</f>
+        <v/>
+      </c>
+      <c r="G6" s="69">
+        <f>F6*0.25</f>
+        <v/>
+      </c>
+      <c r="H6" s="69">
+        <f>F6*0.25</f>
+        <v/>
+      </c>
+      <c r="I6" s="69">
+        <f>F6*0.50</f>
+        <v/>
+      </c>
+      <c r="J6" s="68" t="inlineStr">
+        <is>
+          <t>Ausbezahlt</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="68" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="68" t="inlineStr">
+        <is>
+          <t>Aktuell</t>
+        </is>
+      </c>
+      <c r="C7" s="69" t="n"/>
+      <c r="D7" s="69" t="n"/>
+      <c r="E7" s="68" t="inlineStr"/>
+      <c r="F7" s="69" t="n"/>
+      <c r="G7" s="69" t="n"/>
+      <c r="H7" s="69" t="n"/>
+      <c r="I7" s="69" t="n"/>
+      <c r="J7" s="68" t="inlineStr">
+        <is>
+          <t>Offen (seit 12.05.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="70" t="inlineStr">
+        <is>
+          <t>SUMME</t>
+        </is>
+      </c>
+      <c r="B8" s="68" t="n"/>
+      <c r="C8" s="71">
+        <f>SUM(C2:C7)</f>
+        <v/>
+      </c>
+      <c r="D8" s="71">
+        <f>SUM(D2:D7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="68" t="n"/>
+      <c r="F8" s="71">
+        <f>SUM(F2:F7)</f>
+        <v/>
+      </c>
+      <c r="G8" s="71">
+        <f>SUM(G2:G7)</f>
+        <v/>
+      </c>
+      <c r="H8" s="71">
+        <f>SUM(H2:H7)</f>
+        <v/>
+      </c>
+      <c r="I8" s="71">
+        <f>SUM(I2:I7)</f>
+        <v/>
+      </c>
+      <c r="J8" s="68" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="003B9EFF"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="67" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="B1" s="67" t="inlineStr">
+        <is>
+          <t>Bitget</t>
+        </is>
+      </c>
+      <c r="C1" s="67" t="inlineStr">
+        <is>
+          <t>Phemex</t>
+        </is>
+      </c>
+      <c r="D1" s="67" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="E1" s="67" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="F1" s="67" t="inlineStr">
+        <is>
+          <t>Gesamt</t>
+        </is>
+      </c>
+      <c r="G1" s="67" t="inlineStr">
+        <is>
+          <t>Einzahlungen</t>
+        </is>
+      </c>
+      <c r="H1" s="67" t="inlineStr">
+        <is>
+          <t>Gewinn_Verlust</t>
+        </is>
+      </c>
+      <c r="I1" s="67" t="inlineStr">
+        <is>
+          <t>Kommentar</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="68" t="inlineStr">
+        <is>
+          <t>14.04.2026</t>
+        </is>
+      </c>
+      <c r="B2" s="69" t="n">
+        <v>19542</v>
+      </c>
+      <c r="C2" s="69" t="n">
+        <v>2067</v>
+      </c>
+      <c r="D2" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="69">
+        <f>SUM(B2:E2)</f>
+        <v/>
+      </c>
+      <c r="G2" s="69" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="H2" s="69">
+        <f>F2+G2</f>
+        <v/>
+      </c>
+      <c r="I2" s="68" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="68" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B3" s="69" t="n">
+        <v>20310</v>
+      </c>
+      <c r="C3" s="69" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D3" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="69">
+        <f>SUM(B3:E3)</f>
+        <v/>
+      </c>
+      <c r="G3" s="69" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="H3" s="69">
+        <f>F3+G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="68" t="inlineStr">
+        <is>
+          <t>Angezeigt war 22357, Diff $37 ungeklaert - evtl. Transfer/Fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="68" t="inlineStr">
+        <is>
+          <t>12.05.2026</t>
+        </is>
+      </c>
+      <c r="B4" s="69" t="n">
+        <v>21421</v>
+      </c>
+      <c r="C4" s="69" t="n">
+        <v>1562</v>
+      </c>
+      <c r="D4" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="69">
+        <f>SUM(B4:E4)</f>
+        <v/>
+      </c>
+      <c r="G4" s="69" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="H4" s="69">
+        <f>F4+G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="68" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="68" t="inlineStr">
+        <is>
+          <t>15.06.2026</t>
+        </is>
+      </c>
+      <c r="B5" s="69" t="n"/>
+      <c r="C5" s="69" t="n"/>
+      <c r="D5" s="69" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E5" s="69" t="n">
+        <v>167.85</v>
+      </c>
+      <c r="F5" s="69">
+        <f>SUM(B5:E5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="69" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="H5" s="69">
+        <f>F5+G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="68" t="inlineStr">
+        <is>
+          <t>Bybit: nach Audit-Close, Differenz evtl. durch hohe Fees bei Bot-Trading</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00EF4444"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="67" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="B1" s="67" t="inlineStr">
+        <is>
+          <t>Posten</t>
+        </is>
+      </c>
+      <c r="C1" s="67" t="inlineStr">
+        <is>
+          <t>Betrag</t>
+        </is>
+      </c>
+      <c r="D1" s="67" t="inlineStr">
+        <is>
+          <t>Kategorie</t>
+        </is>
+      </c>
+      <c r="E1" s="67" t="inlineStr">
+        <is>
+          <t>Kommentar</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="68" t="inlineStr">
+        <is>
+          <t>~04.2026</t>
+        </is>
+      </c>
+      <c r="B2" s="68" t="inlineStr">
+        <is>
+          <t>Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="C2" s="69" t="n">
+        <v>100</v>
+      </c>
+      <c r="D2" s="68" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="E2" s="68" t="inlineStr">
+        <is>
+          <t>Datum noch zu bestaetigen</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="68" t="inlineStr">
+        <is>
+          <t>~04.2026</t>
+        </is>
+      </c>
+      <c r="B3" s="68" t="inlineStr">
+        <is>
+          <t>TradingView</t>
+        </is>
+      </c>
+      <c r="C3" s="69" t="n">
+        <v>50</v>
+      </c>
+      <c r="D3" s="68" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="E3" s="68" t="inlineStr">
+        <is>
+          <t>Datum noch zu bestaetigen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="68" t="inlineStr">
+        <is>
+          <t>Geplant</t>
+        </is>
+      </c>
+      <c r="B4" s="68" t="inlineStr">
+        <is>
+          <t>VPS DigitalOcean</t>
+        </is>
+      </c>
+      <c r="C4" s="68" t="inlineStr">
+        <is>
+          <t>6-12/Monat</t>
+        </is>
+      </c>
+      <c r="D4" s="68" t="inlineStr">
+        <is>
+          <t>Infrastruktur</t>
+        </is>
+      </c>
+      <c r="E4" s="68" t="inlineStr">
+        <is>
+          <t>$200 Startguthaben vorhanden</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="72" t="inlineStr">
+        <is>
+          <t>SUMME</t>
+        </is>
+      </c>
+      <c r="C6" s="73">
+        <f>SUM(C2:C3)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00F59E0B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="74" t="inlineStr">
+        <is>
+          <t>Kennzahl</t>
+        </is>
+      </c>
+      <c r="B1" s="74" t="inlineStr">
+        <is>
+          <t>Wert</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="75" t="inlineStr">
+        <is>
+          <t>Total Einzahlungen</t>
+        </is>
+      </c>
+      <c r="B2" s="76" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="75" t="inlineStr">
+        <is>
+          <t>Total Ausbezahlt (Verteilung)</t>
+        </is>
+      </c>
+      <c r="B3" s="76">
+        <f>SUMPRODUCT((Auszahlungen!J2:J7="Ausbezahlt")*Auszahlungen!F2:F7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="75" t="inlineStr">
+        <is>
+          <t>TR Kumuliert</t>
+        </is>
+      </c>
+      <c r="B4" s="76">
+        <f>SUMPRODUCT((Auszahlungen!J2:J7="Ausbezahlt")*Auszahlungen!G2:G7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="75" t="inlineStr">
+        <is>
+          <t>GT Kumuliert</t>
+        </is>
+      </c>
+      <c r="B5" s="76">
+        <f>SUMPRODUCT((Auszahlungen!J2:J7="Ausbezahlt")*Auszahlungen!H2:H7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="75" t="inlineStr">
+        <is>
+          <t>CK Kumuliert</t>
+        </is>
+      </c>
+      <c r="B6" s="76">
+        <f>SUMPRODUCT((Auszahlungen!J2:J7="Ausbezahlt")*Auszahlungen!I2:I7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="75" t="inlineStr">
+        <is>
+          <t>Total Ausgaben</t>
+        </is>
+      </c>
+      <c r="B7" s="76">
+        <f>Ausgaben!C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="75" t="inlineStr">
+        <is>
+          <t>Aktueller Boersenstand</t>
+        </is>
+      </c>
+      <c r="B8" s="76">
+        <f>INDEX(Boersenstand!F2:F100,MATCH(9.99E+307,Boersenstand!F2:F100))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="75" t="inlineStr">
+        <is>
+          <t>Gewinn/Verlust (Boersenstand - Einzahlungen)</t>
+        </is>
+      </c>
+      <c r="B9" s="76">
+        <f>B9-B2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="75" t="inlineStr">
+        <is>
+          <t>ROE TR (auf $10,000)</t>
+        </is>
+      </c>
+      <c r="B10" s="76">
+        <f>B4/10000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="75" t="inlineStr">
+        <is>
+          <t>ROE GT (auf $10,000)</t>
+        </is>
+      </c>
+      <c r="B11" s="77">
+        <f>B5/10000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="78" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>